<commit_message>
fix: a column width is saved and loaded with the padding of the workbook's digit width, not a fixed 96 DPI 0.71 (#803)
The padding is 2 * ceil(mdw / 4) + 1 px of an mdw px digit, scaled below one digit, as Excel 16.0 writes and reads it (measured over COM at 120 DPI). The load takes off the same padding and rounds to the six decimals a save writes, so a width loads back as it was set at any DPI; a loaded width keeps the file's spelling while it loads as the same width. 65 reference files regenerated (col widths only).
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/Columns/ColumnCollection.xlsx
+++ b/XLibur.Tests/Resource/Examples/Columns/ColumnCollection.xlsx
@@ -448,7 +448,7 @@
   <x:dimension ref="A1:V6"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="22" width="3.710625" customWidth="1"/>
+    <x:col min="1" max="22" width="3.714286" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:22">
@@ -520,21 +520,21 @@
   <x:dimension ref="A1"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="2" width="3.710625" style="2" customWidth="1"/>
-    <x:col min="3" max="3" width="3.710625" customWidth="1"/>
-    <x:col min="4" max="5" width="3.710625" style="3" customWidth="1"/>
-    <x:col min="6" max="6" width="3.710625" customWidth="1"/>
-    <x:col min="7" max="8" width="3.710625" style="4" customWidth="1"/>
-    <x:col min="9" max="9" width="3.710625" customWidth="1"/>
-    <x:col min="10" max="11" width="3.710625" style="5" customWidth="1"/>
-    <x:col min="12" max="12" width="3.710625" customWidth="1"/>
-    <x:col min="13" max="14" width="3.710625" style="5" customWidth="1"/>
-    <x:col min="15" max="15" width="3.710625" customWidth="1"/>
-    <x:col min="16" max="17" width="3.710625" style="6" customWidth="1"/>
-    <x:col min="18" max="18" width="3.710625" customWidth="1"/>
-    <x:col min="19" max="20" width="3.710625" style="6" customWidth="1"/>
-    <x:col min="21" max="21" width="3.710625" customWidth="1"/>
-    <x:col min="22" max="22" width="3.710625" style="7" customWidth="1"/>
+    <x:col min="1" max="2" width="3.714286" style="2" customWidth="1"/>
+    <x:col min="3" max="3" width="3.714286" customWidth="1"/>
+    <x:col min="4" max="5" width="3.714286" style="3" customWidth="1"/>
+    <x:col min="6" max="6" width="3.714286" customWidth="1"/>
+    <x:col min="7" max="8" width="3.714286" style="4" customWidth="1"/>
+    <x:col min="9" max="9" width="3.714286" customWidth="1"/>
+    <x:col min="10" max="11" width="3.714286" style="5" customWidth="1"/>
+    <x:col min="12" max="12" width="3.714286" customWidth="1"/>
+    <x:col min="13" max="14" width="3.714286" style="5" customWidth="1"/>
+    <x:col min="15" max="15" width="3.714286" customWidth="1"/>
+    <x:col min="16" max="17" width="3.714286" style="6" customWidth="1"/>
+    <x:col min="18" max="18" width="3.714286" customWidth="1"/>
+    <x:col min="19" max="20" width="3.714286" style="6" customWidth="1"/>
+    <x:col min="21" max="21" width="3.714286" customWidth="1"/>
+    <x:col min="22" max="22" width="3.714286" style="7" customWidth="1"/>
   </x:cols>
   <x:sheetData/>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>